<commit_message>
feat : excel data -> scriptable object data -> addressable load
</commit_message>
<xml_diff>
--- a/Excels/GameData.xlsx
+++ b/Excels/GameData.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Devs\TRPG.Client\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF804BF-B476-4D17-AC18-09E8F6EA19DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B54BC5-C7FF-47C2-8CE2-2D644C056C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4C3ECC9E-3FC4-471E-A1D2-0D99937C0D65}"/>
   </bookViews>
   <sheets>
-    <sheet name="MonsterData" sheetId="1" r:id="rId1"/>
+    <sheet name="CreatureData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Damage</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>쥐</t>
-  </si>
-  <si>
-    <t>PF_Monster_00</t>
   </si>
   <si>
     <t>Attack_00</t>
@@ -75,10 +72,6 @@
   </si>
   <si>
     <t>Hp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PrefabAddress</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -638,33 +631,30 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" thickBot="1">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="18" thickBot="1">
       <c r="A2" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>3</v>
@@ -672,20 +662,17 @@
       <c r="C2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="5">
+        <v>10</v>
+      </c>
+      <c r="E2" s="5">
         <v>5</v>
       </c>
-      <c r="E2" s="5">
-        <v>10</v>
-      </c>
       <c r="F2" s="5">
+        <v>1</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>5</v>
-      </c>
-      <c r="G2" s="5">
-        <v>1</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" thickBot="1">

</xml_diff>

<commit_message>
feat : CRT shader
</commit_message>
<xml_diff>
--- a/Excels/GameData.xlsx
+++ b/Excels/GameData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Devs\TRPG.Client\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B54BC5-C7FF-47C2-8CE2-2D644C056C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0E4C97-7593-4B01-BA53-255D9D666B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4C3ECC9E-3FC4-471E-A1D2-0D99937C0D65}"/>
   </bookViews>
@@ -666,7 +666,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2" s="5">
         <v>1</v>

</xml_diff>